<commit_message>
fix: resolve UnicodeEncodeError in generate_unittest_excel.py and regenerate UnitestKCPM.xlsx with BVA test cases
</commit_message>
<xml_diff>
--- a/UnitestKCPM.xlsx
+++ b/UnitestKCPM.xlsx
@@ -683,7 +683,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -746,7 +746,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -810,7 +810,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -874,7 +874,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -937,7 +937,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1002,7 +1002,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1129,7 +1129,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -1193,7 +1193,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1257,7 +1257,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -1322,7 +1322,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1385,12 +1385,12 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>11A6_03_Đăng</t>
+          <t>Đăng</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1449,12 +1449,12 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>11A6_03_Đăng</t>
+          <t>Đăng</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1512,12 +1512,12 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>11A6_03_Đăng</t>
+          <t>Đăng</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1575,12 +1575,12 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>11A6_03_Đăng</t>
+          <t>Đăng</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1638,12 +1638,12 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>11A6_03_Đăng</t>
+          <t>Đăng</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1701,7 +1701,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1764,7 +1764,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -1827,7 +1827,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -1953,7 +1953,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -2015,7 +2015,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -2079,7 +2079,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -2206,7 +2206,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -2269,7 +2269,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -2332,12 +2332,12 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>11A6_03_Đăng</t>
+          <t>Đăng</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -2396,12 +2396,12 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>11A6_03_Đăng</t>
+          <t>Đăng</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2459,12 +2459,12 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>11A6_03_Đăng</t>
+          <t>Đăng</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -2522,12 +2522,12 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>11A6_03_Đăng</t>
+          <t>Đăng</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -2584,12 +2584,12 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>11A6_03_Đăng</t>
+          <t>Đăng</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -2647,7 +2647,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -2710,7 +2710,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -2773,7 +2773,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -2837,7 +2837,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -2900,7 +2900,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -3026,7 +3026,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -3089,7 +3089,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -3151,7 +3151,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -3215,7 +3215,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -3278,7 +3278,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -3340,7 +3340,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -3404,7 +3404,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -3469,7 +3469,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -3534,7 +3534,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -3662,7 +3662,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -3726,7 +3726,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -3790,7 +3790,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -3854,7 +3854,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -3918,7 +3918,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -3981,7 +3981,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -4044,7 +4044,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -4172,7 +4172,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -4236,7 +4236,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -4300,7 +4300,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -4364,7 +4364,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -4428,7 +4428,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -4491,7 +4491,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -4554,7 +4554,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -4617,7 +4617,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -4680,7 +4680,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -4743,7 +4743,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -4869,7 +4869,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -4932,7 +4932,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -4995,7 +4995,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -5058,7 +5058,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -5122,7 +5122,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -5186,7 +5186,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -5249,7 +5249,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -5312,7 +5312,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -5375,7 +5375,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -5438,7 +5438,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -5501,7 +5501,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -5564,7 +5564,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -5627,7 +5627,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -5690,7 +5690,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -6356,17 +6356,17 @@
       <c r="D25" s="6" t="n"/>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G25" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="H25" s="6" t="n"/>
@@ -7083,17 +7083,17 @@
       <c r="D25" s="6" t="n"/>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G25" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="H25" s="6" t="n"/>
@@ -8150,42 +8150,42 @@
       <c r="D33" s="6" t="n"/>
       <c r="E33" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="F33" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G33" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="H33" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="J33" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="K33" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="L33" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="M33" s="6" t="n"/>
@@ -9193,32 +9193,32 @@
       <c r="D33" s="6" t="n"/>
       <c r="E33" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="F33" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G33" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="H33" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="J33" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="K33" s="6" t="n"/>
@@ -10257,42 +10257,42 @@
       <c r="D33" s="6" t="n"/>
       <c r="E33" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="F33" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G33" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="H33" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="J33" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="K33" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="L33" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="M33" s="6" t="n"/>
@@ -11151,32 +11151,32 @@
       <c r="D28" s="6" t="n"/>
       <c r="E28" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="F28" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G28" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="H28" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="J28" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="K28" s="6" t="n"/>
@@ -12045,32 +12045,32 @@
       <c r="D29" s="6" t="n"/>
       <c r="E29" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="F29" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G29" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="H29" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="J29" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="K29" s="6" t="n"/>
@@ -12988,27 +12988,27 @@
       <c r="D32" s="6" t="n"/>
       <c r="E32" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="F32" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G32" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="H32" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="I32" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="J32" s="6" t="n"/>
@@ -14012,32 +14012,32 @@
       <c r="D33" s="6" t="n"/>
       <c r="E33" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="F33" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G33" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="H33" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="J33" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="K33" s="6" t="n"/>
@@ -14175,7 +14175,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>11A6_03_Đăng</t>
+          <t>Đăng</t>
         </is>
       </c>
       <c r="C3" s="6" t="n"/>
@@ -14191,7 +14191,7 @@
       <c r="I3" s="6" t="n"/>
       <c r="J3" s="7" t="inlineStr">
         <is>
-          <t>11A6_03_Đăng</t>
+          <t>Đăng</t>
         </is>
       </c>
       <c r="K3" s="6" t="n"/>
@@ -14876,27 +14876,27 @@
       <c r="D28" s="6" t="n"/>
       <c r="E28" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="F28" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G28" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="H28" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="J28" s="6" t="n"/>
@@ -15799,32 +15799,32 @@
       <c r="D30" s="6" t="n"/>
       <c r="E30" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="F30" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G30" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="H30" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="J30" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="K30" s="6" t="n"/>
@@ -16603,22 +16603,22 @@
       <c r="D27" s="6" t="n"/>
       <c r="E27" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="F27" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G27" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="H27" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="I27" s="6" t="n"/>
@@ -16754,7 +16754,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>11A6_03_Đăng</t>
+          <t>Đăng</t>
         </is>
       </c>
       <c r="C3" s="6" t="n"/>
@@ -16770,7 +16770,7 @@
       <c r="I3" s="6" t="n"/>
       <c r="J3" s="7" t="inlineStr">
         <is>
-          <t>11A6_03_Đăng</t>
+          <t>Đăng</t>
         </is>
       </c>
       <c r="K3" s="6" t="n"/>
@@ -17511,27 +17511,27 @@
       <c r="D31" s="6" t="n"/>
       <c r="E31" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="F31" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G31" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="H31" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="I31" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="J31" s="6" t="n"/>
@@ -18289,22 +18289,22 @@
       <c r="D26" s="6" t="n"/>
       <c r="E26" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G26" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="H26" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="I26" s="6" t="n"/>
@@ -19198,27 +19198,27 @@
       <c r="D31" s="6" t="n"/>
       <c r="E31" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="F31" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="G31" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="H31" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="I31" s="8" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="J31" s="6" t="n"/>

</xml_diff>